<commit_message>
Bricks Vocabulary 4800 전량 생성 (학생용/정답)
book_name 혼입(Unit 30 'tilt' 1줄: Bricks Vocabulary 30 → 4800) 교정 후
excel/Bricks Vocabulary 4800.xlsx(900단어/30유닛)로 --from 1 --to 30 --answer 실행.
output_new/Bricks Vocabulary 4800/ 아래 학생용·정답 각 374쪽 PDF+HTML. PROGRESS 갱신.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Bricks Vocabulary 4800.xlsx
+++ b/excel/Bricks Vocabulary 4800.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\학원파일\클래스카드 작업용\단어프로그램 작업용 엑셀파일\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ytrbh\Desktop\Vocaworkbook\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5802" uniqueCount="3611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5802" uniqueCount="3610">
   <si>
     <t>book_name</t>
   </si>
@@ -10623,9 +10623,6 @@
   </si>
   <si>
     <t>Parents must consent to this trip.</t>
-  </si>
-  <si>
-    <t>Bricks Vocabulary 30</t>
   </si>
   <si>
     <t>tilt</t>
@@ -11220,7 +11217,8 @@
   <dimension ref="A1:H901"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="21.25" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33119,7 +33117,7 @@
     </row>
     <row r="881" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A881" s="2" t="s">
-        <v>3533</v>
+        <v>8</v>
       </c>
       <c r="B881" s="2" t="s">
         <v>3505</v>
@@ -33128,19 +33126,19 @@
         <v>10</v>
       </c>
       <c r="D881" s="2" t="s">
+        <v>3533</v>
+      </c>
+      <c r="E881" s="2" t="s">
         <v>3534</v>
       </c>
-      <c r="E881" s="2" t="s">
+      <c r="F881" s="2" t="s">
         <v>3535</v>
       </c>
-      <c r="F881" s="2" t="s">
+      <c r="G881" s="2" t="s">
         <v>3536</v>
       </c>
-      <c r="G881" s="2" t="s">
+      <c r="H881" s="1" t="s">
         <v>3537</v>
-      </c>
-      <c r="H881" s="1" t="s">
-        <v>3538</v>
       </c>
     </row>
     <row r="882" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33154,19 +33152,19 @@
         <v>11</v>
       </c>
       <c r="D882" s="2" t="s">
+        <v>3538</v>
+      </c>
+      <c r="E882" s="2" t="s">
         <v>3539</v>
       </c>
-      <c r="E882" s="2" t="s">
+      <c r="F882" s="2" t="s">
         <v>3540</v>
       </c>
-      <c r="F882" s="2" t="s">
+      <c r="G882" s="2" t="s">
         <v>3541</v>
       </c>
-      <c r="G882" s="2" t="s">
+      <c r="H882" s="1" t="s">
         <v>3542</v>
-      </c>
-      <c r="H882" s="1" t="s">
-        <v>3543</v>
       </c>
     </row>
     <row r="883" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33180,17 +33178,17 @@
         <v>12</v>
       </c>
       <c r="D883" s="2" t="s">
+        <v>3543</v>
+      </c>
+      <c r="E883" s="2" t="s">
         <v>3544</v>
       </c>
-      <c r="E883" s="2" t="s">
+      <c r="F883" s="2" t="s">
         <v>3545</v>
-      </c>
-      <c r="F883" s="2" t="s">
-        <v>3546</v>
       </c>
       <c r="G883" s="2"/>
       <c r="H883" s="1" t="s">
-        <v>3547</v>
+        <v>3546</v>
       </c>
     </row>
     <row r="884" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33204,15 +33202,15 @@
         <v>13</v>
       </c>
       <c r="D884" s="2" t="s">
+        <v>3547</v>
+      </c>
+      <c r="E884" s="2" t="s">
         <v>3548</v>
-      </c>
-      <c r="E884" s="2" t="s">
-        <v>3549</v>
       </c>
       <c r="F884" s="2"/>
       <c r="G884" s="2"/>
       <c r="H884" s="1" t="s">
-        <v>3550</v>
+        <v>3549</v>
       </c>
     </row>
     <row r="885" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33226,17 +33224,17 @@
         <v>14</v>
       </c>
       <c r="D885" s="2" t="s">
+        <v>3550</v>
+      </c>
+      <c r="E885" s="2" t="s">
         <v>3551</v>
-      </c>
-      <c r="E885" s="2" t="s">
-        <v>3552</v>
       </c>
       <c r="F885" s="2" t="s">
         <v>232</v>
       </c>
       <c r="G885" s="2"/>
       <c r="H885" s="1" t="s">
-        <v>3553</v>
+        <v>3552</v>
       </c>
     </row>
     <row r="886" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33250,17 +33248,17 @@
         <v>15</v>
       </c>
       <c r="D886" s="2" t="s">
+        <v>3553</v>
+      </c>
+      <c r="E886" s="2" t="s">
         <v>3554</v>
       </c>
-      <c r="E886" s="2" t="s">
+      <c r="F886" s="2" t="s">
         <v>3555</v>
-      </c>
-      <c r="F886" s="2" t="s">
-        <v>3556</v>
       </c>
       <c r="G886" s="2"/>
       <c r="H886" s="1" t="s">
-        <v>3557</v>
+        <v>3556</v>
       </c>
     </row>
     <row r="887" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33274,19 +33272,19 @@
         <v>16</v>
       </c>
       <c r="D887" s="2" t="s">
+        <v>3557</v>
+      </c>
+      <c r="E887" s="2" t="s">
         <v>3558</v>
       </c>
-      <c r="E887" s="2" t="s">
+      <c r="F887" s="2" t="s">
         <v>3559</v>
       </c>
-      <c r="F887" s="2" t="s">
+      <c r="G887" s="2" t="s">
         <v>3560</v>
       </c>
-      <c r="G887" s="2" t="s">
+      <c r="H887" s="1" t="s">
         <v>3561</v>
-      </c>
-      <c r="H887" s="1" t="s">
-        <v>3562</v>
       </c>
     </row>
     <row r="888" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33300,17 +33298,17 @@
         <v>17</v>
       </c>
       <c r="D888" s="2" t="s">
-        <v>3563</v>
+        <v>3562</v>
       </c>
       <c r="E888" s="2" t="s">
         <v>1483</v>
       </c>
       <c r="F888" s="2" t="s">
-        <v>3564</v>
+        <v>3563</v>
       </c>
       <c r="G888" s="2"/>
       <c r="H888" s="1" t="s">
-        <v>3565</v>
+        <v>3564</v>
       </c>
     </row>
     <row r="889" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33324,7 +33322,7 @@
         <v>18</v>
       </c>
       <c r="D889" s="2" t="s">
-        <v>3566</v>
+        <v>3565</v>
       </c>
       <c r="E889" s="2" t="s">
         <v>2214</v>
@@ -33334,7 +33332,7 @@
       </c>
       <c r="G889" s="2"/>
       <c r="H889" s="1" t="s">
-        <v>3567</v>
+        <v>3566</v>
       </c>
     </row>
     <row r="890" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33348,10 +33346,10 @@
         <v>19</v>
       </c>
       <c r="D890" s="2" t="s">
+        <v>3567</v>
+      </c>
+      <c r="E890" s="2" t="s">
         <v>3568</v>
-      </c>
-      <c r="E890" s="2" t="s">
-        <v>3569</v>
       </c>
       <c r="F890" s="2" t="s">
         <v>382</v>
@@ -33360,7 +33358,7 @@
         <v>299</v>
       </c>
       <c r="H890" s="1" t="s">
-        <v>3570</v>
+        <v>3569</v>
       </c>
     </row>
     <row r="891" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33374,17 +33372,17 @@
         <v>20</v>
       </c>
       <c r="D891" s="2" t="s">
+        <v>3570</v>
+      </c>
+      <c r="E891" s="2" t="s">
         <v>3571</v>
       </c>
-      <c r="E891" s="2" t="s">
+      <c r="F891" s="2" t="s">
         <v>3572</v>
-      </c>
-      <c r="F891" s="2" t="s">
-        <v>3573</v>
       </c>
       <c r="G891" s="2"/>
       <c r="H891" s="1" t="s">
-        <v>3574</v>
+        <v>3573</v>
       </c>
     </row>
     <row r="892" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33398,17 +33396,17 @@
         <v>21</v>
       </c>
       <c r="D892" s="2" t="s">
+        <v>3574</v>
+      </c>
+      <c r="E892" s="2" t="s">
         <v>3575</v>
       </c>
-      <c r="E892" s="2" t="s">
+      <c r="F892" s="2" t="s">
         <v>3576</v>
-      </c>
-      <c r="F892" s="2" t="s">
-        <v>3577</v>
       </c>
       <c r="G892" s="2"/>
       <c r="H892" s="1" t="s">
-        <v>3578</v>
+        <v>3577</v>
       </c>
     </row>
     <row r="893" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33422,10 +33420,10 @@
         <v>22</v>
       </c>
       <c r="D893" s="2" t="s">
+        <v>3578</v>
+      </c>
+      <c r="E893" s="2" t="s">
         <v>3579</v>
-      </c>
-      <c r="E893" s="2" t="s">
-        <v>3580</v>
       </c>
       <c r="F893" s="2" t="s">
         <v>2287</v>
@@ -33434,7 +33432,7 @@
         <v>1138</v>
       </c>
       <c r="H893" s="1" t="s">
-        <v>3581</v>
+        <v>3580</v>
       </c>
     </row>
     <row r="894" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33448,19 +33446,19 @@
         <v>23</v>
       </c>
       <c r="D894" s="2" t="s">
+        <v>3581</v>
+      </c>
+      <c r="E894" s="2" t="s">
         <v>3582</v>
       </c>
-      <c r="E894" s="2" t="s">
+      <c r="F894" s="2" t="s">
         <v>3583</v>
       </c>
-      <c r="F894" s="2" t="s">
+      <c r="G894" s="2" t="s">
         <v>3584</v>
       </c>
-      <c r="G894" s="2" t="s">
+      <c r="H894" s="1" t="s">
         <v>3585</v>
-      </c>
-      <c r="H894" s="1" t="s">
-        <v>3586</v>
       </c>
     </row>
     <row r="895" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33474,17 +33472,17 @@
         <v>24</v>
       </c>
       <c r="D895" s="2" t="s">
+        <v>3586</v>
+      </c>
+      <c r="E895" s="2" t="s">
         <v>3587</v>
       </c>
-      <c r="E895" s="2" t="s">
+      <c r="F895" s="2" t="s">
         <v>3588</v>
-      </c>
-      <c r="F895" s="2" t="s">
-        <v>3589</v>
       </c>
       <c r="G895" s="2"/>
       <c r="H895" s="1" t="s">
-        <v>3590</v>
+        <v>3589</v>
       </c>
     </row>
     <row r="896" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33498,17 +33496,17 @@
         <v>25</v>
       </c>
       <c r="D896" s="2" t="s">
+        <v>3590</v>
+      </c>
+      <c r="E896" s="2" t="s">
         <v>3591</v>
       </c>
-      <c r="E896" s="2" t="s">
+      <c r="F896" s="2" t="s">
         <v>3592</v>
-      </c>
-      <c r="F896" s="2" t="s">
-        <v>3593</v>
       </c>
       <c r="G896" s="2"/>
       <c r="H896" s="1" t="s">
-        <v>3594</v>
+        <v>3593</v>
       </c>
     </row>
     <row r="897" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33522,10 +33520,10 @@
         <v>26</v>
       </c>
       <c r="D897" s="2" t="s">
+        <v>3594</v>
+      </c>
+      <c r="E897" s="2" t="s">
         <v>3595</v>
-      </c>
-      <c r="E897" s="2" t="s">
-        <v>3596</v>
       </c>
       <c r="F897" s="2" t="s">
         <v>2918</v>
@@ -33534,7 +33532,7 @@
         <v>2041</v>
       </c>
       <c r="H897" s="1" t="s">
-        <v>3597</v>
+        <v>3596</v>
       </c>
     </row>
     <row r="898" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33548,19 +33546,19 @@
         <v>27</v>
       </c>
       <c r="D898" s="2" t="s">
-        <v>3598</v>
+        <v>3597</v>
       </c>
       <c r="E898" s="2" t="s">
         <v>2598</v>
       </c>
       <c r="F898" s="2" t="s">
-        <v>3599</v>
+        <v>3598</v>
       </c>
       <c r="G898" s="2" t="s">
         <v>741</v>
       </c>
       <c r="H898" s="1" t="s">
-        <v>3600</v>
+        <v>3599</v>
       </c>
     </row>
     <row r="899" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33574,19 +33572,19 @@
         <v>28</v>
       </c>
       <c r="D899" s="2" t="s">
+        <v>3600</v>
+      </c>
+      <c r="E899" s="2" t="s">
         <v>3601</v>
       </c>
-      <c r="E899" s="2" t="s">
+      <c r="F899" s="2" t="s">
         <v>3602</v>
-      </c>
-      <c r="F899" s="2" t="s">
-        <v>3603</v>
       </c>
       <c r="G899" s="2" t="s">
         <v>150</v>
       </c>
       <c r="H899" s="1" t="s">
-        <v>3604</v>
+        <v>3603</v>
       </c>
     </row>
     <row r="900" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33600,17 +33598,17 @@
         <v>29</v>
       </c>
       <c r="D900" s="2" t="s">
+        <v>3604</v>
+      </c>
+      <c r="E900" s="2" t="s">
         <v>3605</v>
       </c>
-      <c r="E900" s="2" t="s">
+      <c r="F900" s="2" t="s">
         <v>3606</v>
-      </c>
-      <c r="F900" s="2" t="s">
-        <v>3607</v>
       </c>
       <c r="G900" s="2"/>
       <c r="H900" s="1" t="s">
-        <v>3608</v>
+        <v>3607</v>
       </c>
     </row>
     <row r="901" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -33624,7 +33622,7 @@
         <v>30</v>
       </c>
       <c r="D901" s="2" t="s">
-        <v>3609</v>
+        <v>3608</v>
       </c>
       <c r="E901" s="2" t="s">
         <v>2627</v>
@@ -33634,7 +33632,7 @@
       </c>
       <c r="G901" s="2"/>
       <c r="H901" s="1" t="s">
-        <v>3610</v>
+        <v>3609</v>
       </c>
     </row>
   </sheetData>

</xml_diff>